<commit_message>
fix: enforce truthful report scope and audit
</commit_message>
<xml_diff>
--- a/07_自动维护工作流/templates/daily_review.xlsx
+++ b/07_自动维护工作流/templates/daily_review.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R9dbd9a24b48f4fe7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行概览" sheetId="2" r:id="Rea3da1d8b5434167"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录变化" sheetId="3" r:id="R16c4c24334814419"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增正式推荐" sheetId="4" r:id="R27c074c9daef47ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本更新" sheetId="5" r:id="Rd7e6811cd4514678"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发现更新未升级" sheetId="6" r:id="R0e0c71a6930d48af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="条件候选" sheetId="7" r:id="Rc31a7b97281b4fdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需适配候选" sheetId="8" r:id="Rea2ebb74bb1c4b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="去重与来源别名" sheetId="9" r:id="Rdfd9650da5994e3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="受影响专业类" sheetId="10" r:id="R9fd831f4db6e4b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排除原因汇总" sheetId="11" r:id="R4c65a99551074ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源请求审计" sheetId="12" r:id="Rfe93d2f8502246a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R0d755fec83fd41c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="执行概览" sheetId="2" r:id="Ra08582f1f03545fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目录变化" sheetId="3" r:id="Rab152fe85681433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增正式推荐" sheetId="4" r:id="Rfa7118492af94980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本更新" sheetId="5" r:id="R2b56b0f22d5d4d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发现更新未升级" sheetId="6" r:id="R188d751d90f34a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="条件候选" sheetId="7" r:id="R80cc9e545994474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需适配候选" sheetId="8" r:id="R2c07288648364a3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="去重与来源别名" sheetId="9" r:id="Rbdc96b35bda7481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="受影响专业类" sheetId="10" r:id="Rd10214ba24764b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="排除原因汇总" sheetId="11" r:id="R0596d0b69e6047c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源请求审计" sheetId="12" r:id="Ra148624e78c746e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -234,13 +234,19 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="DailySourceAudit" displayName="DailySourceAudit" ref="A1:D2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:D2"/>
-  <x:tableColumns count="4">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="DailySourceAudit" displayName="DailySourceAudit" ref="A1:J2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:J2"/>
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="来源平台"/>
     <x:tableColumn id="2" name="请求地址"/>
-    <x:tableColumn id="3" name="状态"/>
-    <x:tableColumn id="4" name="请求时间"/>
+    <x:tableColumn id="3" name="查询标识"/>
+    <x:tableColumn id="4" name="页码"/>
+    <x:tableColumn id="5" name="状态码"/>
+    <x:tableColumn id="6" name="尝试次数"/>
+    <x:tableColumn id="7" name="响应SHA-256"/>
+    <x:tableColumn id="8" name="证据位置"/>
+    <x:tableColumn id="9" name="完成"/>
+    <x:tableColumn id="10" name="请求时间"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -269,9 +275,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DailyFormalAdditions" displayName="DailyFormalAdditions" ref="A1:N2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N2"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="DailyFormalAdditions" displayName="DailyFormalAdditions" ref="A1:P2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P2"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="内部标识"/>
     <x:tableColumn id="2" name="英文原名"/>
     <x:tableColumn id="3" name="规范名称"/>
@@ -286,15 +292,17 @@
     <x:tableColumn id="12" name="限制"/>
     <x:tableColumn id="13" name="专业类"/>
     <x:tableColumn id="14" name="收集日期"/>
+    <x:tableColumn id="15" name="层级"/>
+    <x:tableColumn id="16" name="原因/结论"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DailyVersionUpdates" displayName="DailyVersionUpdates" ref="A1:N2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N2"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="DailyVersionUpdates" displayName="DailyVersionUpdates" ref="A1:P2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P2"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="内部标识"/>
     <x:tableColumn id="2" name="英文原名"/>
     <x:tableColumn id="3" name="规范名称"/>
@@ -309,15 +317,17 @@
     <x:tableColumn id="12" name="限制"/>
     <x:tableColumn id="13" name="专业类"/>
     <x:tableColumn id="14" name="收集日期"/>
+    <x:tableColumn id="15" name="层级"/>
+    <x:tableColumn id="16" name="原因/结论"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DailyUpdatesNotApplied" displayName="DailyUpdatesNotApplied" ref="A1:N2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N2"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="DailyUpdatesNotApplied" displayName="DailyUpdatesNotApplied" ref="A1:P2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P2"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="内部标识"/>
     <x:tableColumn id="2" name="英文原名"/>
     <x:tableColumn id="3" name="规范名称"/>
@@ -332,15 +342,17 @@
     <x:tableColumn id="12" name="限制"/>
     <x:tableColumn id="13" name="专业类"/>
     <x:tableColumn id="14" name="收集日期"/>
+    <x:tableColumn id="15" name="层级"/>
+    <x:tableColumn id="16" name="原因/结论"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DailyConditionalCandidates" displayName="DailyConditionalCandidates" ref="A1:N2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N2"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DailyConditionalCandidates" displayName="DailyConditionalCandidates" ref="A1:P2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P2"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="内部标识"/>
     <x:tableColumn id="2" name="英文原名"/>
     <x:tableColumn id="3" name="规范名称"/>
@@ -355,15 +367,17 @@
     <x:tableColumn id="12" name="限制"/>
     <x:tableColumn id="13" name="专业类"/>
     <x:tableColumn id="14" name="收集日期"/>
+    <x:tableColumn id="15" name="层级"/>
+    <x:tableColumn id="16" name="原因/结论"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DailyAdaptationCandidates" displayName="DailyAdaptationCandidates" ref="A1:N2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:N2"/>
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DailyAdaptationCandidates" displayName="DailyAdaptationCandidates" ref="A1:P2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:P2"/>
+  <x:tableColumns count="16">
     <x:tableColumn id="1" name="内部标识"/>
     <x:tableColumn id="2" name="英文原名"/>
     <x:tableColumn id="3" name="规范名称"/>
@@ -378,6 +392,8 @@
     <x:tableColumn id="12" name="限制"/>
     <x:tableColumn id="13" name="专业类"/>
     <x:tableColumn id="14" name="收集日期"/>
+    <x:tableColumn id="15" name="层级"/>
+    <x:tableColumn id="16" name="原因/结论"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -657,7 +673,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R054efe73ddc04c19"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfb7828487c5424e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -685,7 +701,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb5e21e798474f26"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44783ef706b349f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -713,7 +729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5528af1f9ea045bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59560522285040b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -722,10 +738,16 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -736,9 +758,27 @@
         <x:v>请求地址</x:v>
       </x:c>
       <x:c r="C1" s="27" t="str">
-        <x:v>状态</x:v>
-      </x:c>
-      <x:c r="D1" s="8" t="str">
+        <x:v>查询标识</x:v>
+      </x:c>
+      <x:c r="D1" s="27" t="str">
+        <x:v>页码</x:v>
+      </x:c>
+      <x:c r="E1" s="27" t="str">
+        <x:v>状态码</x:v>
+      </x:c>
+      <x:c r="F1" s="27" t="str">
+        <x:v>尝试次数</x:v>
+      </x:c>
+      <x:c r="G1" s="27" t="str">
+        <x:v>响应SHA-256</x:v>
+      </x:c>
+      <x:c r="H1" s="27" t="str">
+        <x:v>证据位置</x:v>
+      </x:c>
+      <x:c r="I1" s="27" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="J1" s="8" t="str">
         <x:v>请求时间</x:v>
       </x:c>
     </x:row>
@@ -746,12 +786,18 @@
       <x:c r="A2" s="24" t="str"/>
       <x:c r="B2" s="24" t="str"/>
       <x:c r="C2" s="24" t="str"/>
-      <x:c r="D2" s="28" t="str"/>
+      <x:c r="D2" s="29" t="str"/>
+      <x:c r="E2" s="29" t="str"/>
+      <x:c r="F2" s="29" t="str"/>
+      <x:c r="G2" s="24" t="str"/>
+      <x:c r="H2" s="24" t="str"/>
+      <x:c r="I2" s="29" t="str"/>
+      <x:c r="J2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc35e422925d9468f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d9bf975087430d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -777,7 +823,7 @@
         <x:v>运行标识</x:v>
       </x:c>
       <x:c r="B2" s="16" t="str">
-        <x:v>TEMPLATE</x:v>
+        <x:v>template</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
@@ -785,7 +831,7 @@
         <x:v>生成时间</x:v>
       </x:c>
       <x:c r="B3" s="19" t="n">
-        <x:v>46023</x:v>
+        <x:v>46262</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
@@ -848,7 +894,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73741f7dff324c02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R135a0d3bf3e7422f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -876,7 +922,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01ffaf6a6e9e475d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc99d57b0071a4abf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -899,6 +945,8 @@
     <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -941,8 +989,14 @@
       <x:c r="M1" s="27" t="str">
         <x:v>专业类</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>收集日期</x:v>
+      </x:c>
+      <x:c r="O1" s="27" t="str">
+        <x:v>层级</x:v>
+      </x:c>
+      <x:c r="P1" s="8" t="str">
+        <x:v>原因/结论</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
@@ -960,11 +1014,13 @@
       <x:c r="L2" s="24" t="str"/>
       <x:c r="M2" s="24" t="str"/>
       <x:c r="N2" s="30" t="str"/>
+      <x:c r="O2" s="24" t="str"/>
+      <x:c r="P2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94c6c04390c44c11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73d34b86603e470b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -987,6 +1043,8 @@
     <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1029,8 +1087,14 @@
       <x:c r="M1" s="27" t="str">
         <x:v>专业类</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>收集日期</x:v>
+      </x:c>
+      <x:c r="O1" s="27" t="str">
+        <x:v>层级</x:v>
+      </x:c>
+      <x:c r="P1" s="8" t="str">
+        <x:v>原因/结论</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
@@ -1048,11 +1112,13 @@
       <x:c r="L2" s="24" t="str"/>
       <x:c r="M2" s="24" t="str"/>
       <x:c r="N2" s="30" t="str"/>
+      <x:c r="O2" s="24" t="str"/>
+      <x:c r="P2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02dd8eb5fa64444a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc88b04f476954207"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1075,6 +1141,8 @@
     <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1117,8 +1185,14 @@
       <x:c r="M1" s="27" t="str">
         <x:v>专业类</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>收集日期</x:v>
+      </x:c>
+      <x:c r="O1" s="27" t="str">
+        <x:v>层级</x:v>
+      </x:c>
+      <x:c r="P1" s="8" t="str">
+        <x:v>原因/结论</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
@@ -1136,11 +1210,13 @@
       <x:c r="L2" s="24" t="str"/>
       <x:c r="M2" s="24" t="str"/>
       <x:c r="N2" s="30" t="str"/>
+      <x:c r="O2" s="24" t="str"/>
+      <x:c r="P2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ece91a489974108"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra228dd18eca44266"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1163,6 +1239,8 @@
     <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1205,8 +1283,14 @@
       <x:c r="M1" s="27" t="str">
         <x:v>专业类</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>收集日期</x:v>
+      </x:c>
+      <x:c r="O1" s="27" t="str">
+        <x:v>层级</x:v>
+      </x:c>
+      <x:c r="P1" s="8" t="str">
+        <x:v>原因/结论</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
@@ -1224,11 +1308,13 @@
       <x:c r="L2" s="24" t="str"/>
       <x:c r="M2" s="24" t="str"/>
       <x:c r="N2" s="30" t="str"/>
+      <x:c r="O2" s="24" t="str"/>
+      <x:c r="P2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8931292a8054c0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ef81da11df74eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1251,6 +1337,8 @@
     <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1293,8 +1381,14 @@
       <x:c r="M1" s="27" t="str">
         <x:v>专业类</x:v>
       </x:c>
-      <x:c r="N1" s="8" t="str">
+      <x:c r="N1" s="27" t="str">
         <x:v>收集日期</x:v>
+      </x:c>
+      <x:c r="O1" s="27" t="str">
+        <x:v>层级</x:v>
+      </x:c>
+      <x:c r="P1" s="8" t="str">
+        <x:v>原因/结论</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
@@ -1312,11 +1406,13 @@
       <x:c r="L2" s="24" t="str"/>
       <x:c r="M2" s="24" t="str"/>
       <x:c r="N2" s="30" t="str"/>
+      <x:c r="O2" s="24" t="str"/>
+      <x:c r="P2" s="24" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b15f162fa154458"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2526a35274e44501"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1369,7 +1465,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53507cb379c24afb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d6aea8d22514943"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>